<commit_message>
Draft overview feature of ATM
</commit_message>
<xml_diff>
--- a/C/Project/ATM_Sim/Doc/Requirement.xlsx
+++ b/C/Project/ATM_Sim/Doc/Requirement.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Embedded\C\Project\ATM_Sim\Doc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Jira project\Embedded\C\Project\ATM_Sim\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67620170-457A-47F5-9354-6ACE4B6C92CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FF789CA-DEA9-4066-8EA1-F7E2077DC1CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="10170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Requirement" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
   <si>
     <t>SYS</t>
   </si>
@@ -66,16 +66,52 @@
   <si>
     <t>Source code based on C language,
 without UI support capability</t>
+  </si>
+  <si>
+    <t>SYS_003</t>
+  </si>
+  <si>
+    <t>SYS_004</t>
+  </si>
+  <si>
+    <t>SYS_005</t>
+  </si>
+  <si>
+    <t>SYS_006</t>
+  </si>
+  <si>
+    <t>SYS_007</t>
+  </si>
+  <si>
+    <t>ATM appllication should have PIN code</t>
+  </si>
+  <si>
+    <t>ATM appllication should balance view</t>
+  </si>
+  <si>
+    <t>ATM appllication should withdraw money</t>
+  </si>
+  <si>
+    <t>ATM appllication should transfer money</t>
+  </si>
+  <si>
+    <t>ATM appllication should logged in account</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -386,7 +422,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14.453125" bestFit="1" customWidth="1"/>
@@ -428,7 +464,48 @@
         <v>12</v>
       </c>
     </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" t="s">
+        <v>22</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Revert "Draft overview feature of ATM"
This reverts commit 77032a2e7dfdfc10abca2687ffd7c77992a5f9cb.
</commit_message>
<xml_diff>
--- a/C/Project/ATM_Sim/Doc/Requirement.xlsx
+++ b/C/Project/ATM_Sim/Doc/Requirement.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Jira project\Embedded\C\Project\ATM_Sim\Doc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Embedded\C\Project\ATM_Sim\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FF789CA-DEA9-4066-8EA1-F7E2077DC1CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67620170-457A-47F5-9354-6ACE4B6C92CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="10170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Requirement" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>SYS</t>
   </si>
@@ -67,51 +67,15 @@
     <t>Source code based on C language,
 without UI support capability</t>
   </si>
-  <si>
-    <t>SYS_003</t>
-  </si>
-  <si>
-    <t>SYS_004</t>
-  </si>
-  <si>
-    <t>SYS_005</t>
-  </si>
-  <si>
-    <t>SYS_006</t>
-  </si>
-  <si>
-    <t>SYS_007</t>
-  </si>
-  <si>
-    <t>ATM appllication should have PIN code</t>
-  </si>
-  <si>
-    <t>ATM appllication should balance view</t>
-  </si>
-  <si>
-    <t>ATM appllication should withdraw money</t>
-  </si>
-  <si>
-    <t>ATM appllication should transfer money</t>
-  </si>
-  <si>
-    <t>ATM appllication should logged in account</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -422,7 +386,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14.453125" bestFit="1" customWidth="1"/>
@@ -464,48 +428,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>13</v>
-      </c>
-      <c r="B4" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B5" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B6" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>16</v>
-      </c>
-      <c r="B7" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>17</v>
-      </c>
-      <c r="B8" t="s">
-        <v>22</v>
-      </c>
-    </row>
   </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add draft requirement for Cash withdrawl
</commit_message>
<xml_diff>
--- a/C/Project/ATM_Sim/Doc/Requirement.xlsx
+++ b/C/Project/ATM_Sim/Doc/Requirement.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Embedded\C\Project\ATM_Sim\Doc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Jira project\Embedded\C\Project\ATM_Sim\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67620170-457A-47F5-9354-6ACE4B6C92CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DBC436F-E34A-4490-A031-E47AFBF80BBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Requirement" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
   <si>
     <t>SYS</t>
   </si>
@@ -64,18 +64,92 @@
     <t>ATM application should be run console, not using UI</t>
   </si>
   <si>
-    <t>Source code based on C language,
-without UI support capability</t>
+    <t>SYS_003</t>
+  </si>
+  <si>
+    <t>SYS_004</t>
+  </si>
+  <si>
+    <t>Source code based on C language, without UI support capability</t>
+  </si>
+  <si>
+    <t>ATM application will allow user to select the cash withdrawl function</t>
+  </si>
+  <si>
+    <t>ATM application will allow user enter or select the amount of cash to withdraw</t>
+  </si>
+  <si>
+    <t>ATM application will verify that the withdrawl amount does not exceed the available account balance</t>
+  </si>
+  <si>
+    <t>ATM application will dispense the request amount when the withdrawl transaction is successful</t>
+  </si>
+  <si>
+    <t>ATM application will update the account balance after a successful cash withdrawl</t>
+  </si>
+  <si>
+    <t>ATM application will display an error message when the withdrawl amount exceeds the available account balance</t>
+  </si>
+  <si>
+    <t>ATM application will display the current transaction status after each withdrawl operation</t>
+  </si>
+  <si>
+    <t>SYS_005</t>
+  </si>
+  <si>
+    <t>SYS_006</t>
+  </si>
+  <si>
+    <t>SYS_007</t>
+  </si>
+  <si>
+    <t>SYS_008</t>
+  </si>
+  <si>
+    <t>SYS_009</t>
+  </si>
+  <si>
+    <t>ATM application will allow user to cancel the withdrawl transaction before cash is dispensed</t>
+  </si>
+  <si>
+    <t>ATM application will display the result of the withdrawll transaction after processing</t>
+  </si>
+  <si>
+    <t>SYS_010</t>
+  </si>
+  <si>
+    <t>SYS_011</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -101,10 +175,25 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -386,49 +475,139 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="14.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="73.6328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="29.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.36328125" customWidth="1"/>
+    <col min="1" max="1" width="14.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="55.1796875" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="45.90625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="14.36328125" style="1" customWidth="1"/>
+    <col min="5" max="16384" width="8.7265625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
+    <row r="1" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="5" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+    <row r="2" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="29" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
+      <c r="A3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
         <v>12</v>
       </c>
+      <c r="B4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="3"/>
+      <c r="D4" s="4"/>
+    </row>
+    <row r="5" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="3"/>
+      <c r="D5" s="4"/>
+    </row>
+    <row r="6" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="3"/>
+      <c r="D6" s="4"/>
+    </row>
+    <row r="7" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="3"/>
+      <c r="D7" s="4"/>
+    </row>
+    <row r="8" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" s="3"/>
+      <c r="D8" s="4"/>
+    </row>
+    <row r="9" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A9" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9" s="3"/>
+      <c r="D9" s="4"/>
+    </row>
+    <row r="10" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A10" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C10" s="3"/>
+      <c r="D10" s="4"/>
+    </row>
+    <row r="11" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A11" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C11" s="3"/>
+      <c r="D11" s="4"/>
+    </row>
+    <row r="12" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A12" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>28</v>
+      </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
ATM-6 Update Draft define Functional Requirements for Cash Withdrawal
</commit_message>
<xml_diff>
--- a/C/Project/ATM_Sim/Doc/Requirement.xlsx
+++ b/C/Project/ATM_Sim/Doc/Requirement.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Jira project\Embedded\C\Project\ATM_Sim\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DBC436F-E34A-4490-A031-E47AFBF80BBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{635EF8C0-55AA-43AE-A08C-9CF0B7B6857C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="214">
   <si>
     <t>SYS</t>
   </si>
@@ -119,13 +119,573 @@
   </si>
   <si>
     <t>SYS_011</t>
+  </si>
+  <si>
+    <t>LOG_001</t>
+  </si>
+  <si>
+    <t>PIN Authentication</t>
+  </si>
+  <si>
+    <t>LOG_002</t>
+  </si>
+  <si>
+    <t>LOG_003</t>
+  </si>
+  <si>
+    <t>Successful authentication</t>
+  </si>
+  <si>
+    <t>LOG_004</t>
+  </si>
+  <si>
+    <t>Failed authentication</t>
+  </si>
+  <si>
+    <t>LOG_005</t>
+  </si>
+  <si>
+    <t>Retry</t>
+  </si>
+  <si>
+    <t>LOG_006</t>
+  </si>
+  <si>
+    <t>Security</t>
+  </si>
+  <si>
+    <t>LOG_007</t>
+  </si>
+  <si>
+    <t>ATM application will require the user to enter a PIN after inserting a valid card</t>
+  </si>
+  <si>
+    <t>ATM application will verify the entered PIN against the PIN associated with the user's account</t>
+  </si>
+  <si>
+    <t>ATM application will allow the user to retry PIN entry after an incorrect PIN</t>
+  </si>
+  <si>
+    <t>ATM application will terminate the session or block further authentication attempts when the maximum number of incorrect PIN attempts is reached</t>
+  </si>
+  <si>
+    <t>ATM application will allow the user to access ATM services when the PIN is correct</t>
+  </si>
+  <si>
+    <t>ATM application will reject the login attempt when the PIN is incorrect</t>
+  </si>
+  <si>
+    <t>CI_001</t>
+  </si>
+  <si>
+    <t>CI_002</t>
+  </si>
+  <si>
+    <t>CI_003</t>
+  </si>
+  <si>
+    <t>CI_004</t>
+  </si>
+  <si>
+    <t>CI_005</t>
+  </si>
+  <si>
+    <t>ATM  application will not display the entered PIN in plain text on the console</t>
+  </si>
+  <si>
+    <t>ATM application will simulate card insertion when the user starts a transaction</t>
+  </si>
+  <si>
+    <t>ATM application will validate the simulated card before proceeding</t>
+  </si>
+  <si>
+    <t>ATM application will reject an invalid or unsupported card</t>
+  </si>
+  <si>
+    <t>ATM application will proceed to PIN authentication after a valid card is detected</t>
+  </si>
+  <si>
+    <t>ATM  application will simulate returning the card when the transaction is completed or cancelled</t>
+  </si>
+  <si>
+    <t>BI_001</t>
+  </si>
+  <si>
+    <t>BI_002</t>
+  </si>
+  <si>
+    <t>BI_003</t>
+  </si>
+  <si>
+    <t>BI_004</t>
+  </si>
+  <si>
+    <t>ATM application will allow an authenticated user to select the Balance Inquiry function</t>
+  </si>
+  <si>
+    <t>ATM application will retrieve the current balance from the simulated account</t>
+  </si>
+  <si>
+    <t>ATM application will display the current account balance on the console</t>
+  </si>
+  <si>
+    <t>ATM application will allow the user to return to the main menu after viewing the balance</t>
+  </si>
+  <si>
+    <t>CD_001</t>
+  </si>
+  <si>
+    <t>CD_002</t>
+  </si>
+  <si>
+    <t>CD_003</t>
+  </si>
+  <si>
+    <t>CD_004</t>
+  </si>
+  <si>
+    <t>CD_005</t>
+  </si>
+  <si>
+    <t>CD_006</t>
+  </si>
+  <si>
+    <t>Error handling</t>
+  </si>
+  <si>
+    <t>CD_007</t>
+  </si>
+  <si>
+    <t>BI</t>
+  </si>
+  <si>
+    <t>Balance Inquiry</t>
+  </si>
+  <si>
+    <t>CI</t>
+  </si>
+  <si>
+    <t>Card Insertion</t>
+  </si>
+  <si>
+    <t>CD</t>
+  </si>
+  <si>
+    <t>Card Deposit</t>
+  </si>
+  <si>
+    <t>ATM application will allow an authenticated user to select the Cash Deposit function</t>
+  </si>
+  <si>
+    <t>ATM application will allow user to enter the amount of cash to deposited</t>
+  </si>
+  <si>
+    <t>ATM application will reject a deposit amount that is zero or negative</t>
+  </si>
+  <si>
+    <t>ATM application will add the valid deposit amount to the user's account balance</t>
+  </si>
+  <si>
+    <t>ATM application will display the updated account balance after a successful deposit</t>
+  </si>
+  <si>
+    <t>ATM application will display an error message when the deposit amount is invalid</t>
+  </si>
+  <si>
+    <t>ATM application will allow the user to cancel the deposit before confirming the transaction</t>
+  </si>
+  <si>
+    <t>MT_001</t>
+  </si>
+  <si>
+    <t>Money Transfer</t>
+  </si>
+  <si>
+    <t>MT_002</t>
+  </si>
+  <si>
+    <t>MT_003</t>
+  </si>
+  <si>
+    <t>MT_004</t>
+  </si>
+  <si>
+    <t>MT_005</t>
+  </si>
+  <si>
+    <t>MT_006</t>
+  </si>
+  <si>
+    <t>MT_007</t>
+  </si>
+  <si>
+    <t>MT_008</t>
+  </si>
+  <si>
+    <t>MT_009</t>
+  </si>
+  <si>
+    <t>MT_010</t>
+  </si>
+  <si>
+    <t>MT_011</t>
+  </si>
+  <si>
+    <t>MT_012</t>
+  </si>
+  <si>
+    <t>MT_013</t>
+  </si>
+  <si>
+    <t>ATM application will allow an authenticated user to select the Money Transfer function</t>
+  </si>
+  <si>
+    <t>ATM application will allow the user to enter the destination account number</t>
+  </si>
+  <si>
+    <t>ATM application will validate the destination account number before processing the transfer</t>
+  </si>
+  <si>
+    <t>ATM application will allow the user to enter the amount to be transferred</t>
+  </si>
+  <si>
+    <t>ATM application will validate the transfer amount before processing the transaction</t>
+  </si>
+  <si>
+    <t>ATM application will verify that the user's account has sufficient balance for the transfer</t>
+  </si>
+  <si>
+    <t>ATM application will transfer the specified amount from the user's account to the destination account when all validations are successful</t>
+  </si>
+  <si>
+    <t>ATM application will deduct the transferred amount from the user's account after a successful transfer</t>
+  </si>
+  <si>
+    <t>ATM application will add the transferred amount to the destination account after a successful transfer</t>
+  </si>
+  <si>
+    <t>ATM application will display the transfer result to the user after processing the transaction</t>
+  </si>
+  <si>
+    <t>ATM application will display an error message when the destination account is invalid</t>
+  </si>
+  <si>
+    <t>ATM application will display an error message when the user's account has insufficient balance</t>
+  </si>
+  <si>
+    <t>ATM application will allow the user to cancel the transfer before confirmation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MT </t>
+  </si>
+  <si>
+    <t>CP</t>
+  </si>
+  <si>
+    <t>Change PIN</t>
+  </si>
+  <si>
+    <t>TH</t>
+  </si>
+  <si>
+    <t>Transaction History</t>
+  </si>
+  <si>
+    <t>RC</t>
+  </si>
+  <si>
+    <t>Receipt</t>
+  </si>
+  <si>
+    <t>CE</t>
+  </si>
+  <si>
+    <t>Card Ejection</t>
+  </si>
+  <si>
+    <t>TC</t>
+  </si>
+  <si>
+    <t>Transaction Cancellation</t>
+  </si>
+  <si>
+    <t>EH</t>
+  </si>
+  <si>
+    <t>Error Handling</t>
+  </si>
+  <si>
+    <t>Navigation / Main Menu</t>
+  </si>
+  <si>
+    <r>
+      <t>NM</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF0D0D0D"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t>CP_001</t>
+  </si>
+  <si>
+    <t>CP_002</t>
+  </si>
+  <si>
+    <t>CP_003</t>
+  </si>
+  <si>
+    <t>CP_004</t>
+  </si>
+  <si>
+    <t>CP_005</t>
+  </si>
+  <si>
+    <t>CP_006</t>
+  </si>
+  <si>
+    <t>CP_007</t>
+  </si>
+  <si>
+    <t>CP_008</t>
+  </si>
+  <si>
+    <t>TH_001</t>
+  </si>
+  <si>
+    <t>TH_002</t>
+  </si>
+  <si>
+    <t>TH_003</t>
+  </si>
+  <si>
+    <t>TH_004</t>
+  </si>
+  <si>
+    <t>TH_005</t>
+  </si>
+  <si>
+    <t>RC_001</t>
+  </si>
+  <si>
+    <t>RC_002</t>
+  </si>
+  <si>
+    <t>RC_003</t>
+  </si>
+  <si>
+    <t>RC_004</t>
+  </si>
+  <si>
+    <t>RC_005</t>
+  </si>
+  <si>
+    <t>CE_001</t>
+  </si>
+  <si>
+    <t>CE_002</t>
+  </si>
+  <si>
+    <t>CE_003</t>
+  </si>
+  <si>
+    <t>CE_004</t>
+  </si>
+  <si>
+    <t>TC_001</t>
+  </si>
+  <si>
+    <t>TC_002</t>
+  </si>
+  <si>
+    <t>TC_003</t>
+  </si>
+  <si>
+    <t>TC_004</t>
+  </si>
+  <si>
+    <t>TC_005</t>
+  </si>
+  <si>
+    <t>EH_001</t>
+  </si>
+  <si>
+    <t>EH_002</t>
+  </si>
+  <si>
+    <t>EH_003</t>
+  </si>
+  <si>
+    <t>EH_004</t>
+  </si>
+  <si>
+    <t>EH_005</t>
+  </si>
+  <si>
+    <t>EH_006</t>
+  </si>
+  <si>
+    <t>NM_001</t>
+  </si>
+  <si>
+    <t>Main Menu</t>
+  </si>
+  <si>
+    <t>NM_002</t>
+  </si>
+  <si>
+    <t>NM_003</t>
+  </si>
+  <si>
+    <t>NM_004</t>
+  </si>
+  <si>
+    <t>NM_005</t>
+  </si>
+  <si>
+    <t>NM_006</t>
+  </si>
+  <si>
+    <t>NM_007</t>
+  </si>
+  <si>
+    <t>ATM application will allow an authenticated user to select the Change PIN function</t>
+  </si>
+  <si>
+    <t>ATM application will require the user to enter the current PIN before changing the PIN</t>
+  </si>
+  <si>
+    <t>ATM application will verify that the entered current PIN is correct</t>
+  </si>
+  <si>
+    <t>ATM application will require the user to confirm the new PIN</t>
+  </si>
+  <si>
+    <t>ATM application will verify that the new PIN and confirmation PIN match</t>
+  </si>
+  <si>
+    <t>ATM application will update the user's PIN when the new PIN is valid and confirmed</t>
+  </si>
+  <si>
+    <t>ATM application will display an error message when the current PIN is incorrect or the new PIN is invalid</t>
+  </si>
+  <si>
+    <t>ATM application will allow an authenticated user to select the Transaction History function</t>
+  </si>
+  <si>
+    <t>ATM application will retrieve the user's transaction history</t>
+  </si>
+  <si>
+    <t>The transaction history will include the transaction type, amount, and transaction result</t>
+  </si>
+  <si>
+    <t>ATM application will display a message when there are no transaction records available</t>
+  </si>
+  <si>
+    <t>ATM application will allow the user to request a transaction receipt after a completed transaction</t>
+  </si>
+  <si>
+    <t>The receipt will include the transaction type, transaction amount, transaction result, and account balance when applicable</t>
+  </si>
+  <si>
+    <t>ATM application will allow the user to choose whether to receive a receipt after a completed transaction</t>
+  </si>
+  <si>
+    <t>ATM application will not generate a receipt when the user declines the receipt option</t>
+  </si>
+  <si>
+    <t>ATM application will allow the user to end the session and request card ejection</t>
+  </si>
+  <si>
+    <t>ATM application will return the card after a transaction is completed or cancelled</t>
+  </si>
+  <si>
+    <t>ATM application will terminate the current session after the card is returned</t>
+  </si>
+  <si>
+    <t>ATM application will allow the user to cancel an ongoing transaction before confirmation</t>
+  </si>
+  <si>
+    <t>ATM application will terminate the current transaction when the user selects Cancel</t>
+  </si>
+  <si>
+    <t>ATM application will not modify the account balance when a transaction is cancelled before completion</t>
+  </si>
+  <si>
+    <t>ATM application will display a transaction cancellation message to the user</t>
+  </si>
+  <si>
+    <t>ATM application will return the user to the main menu after a transaction is cancelled</t>
+  </si>
+  <si>
+    <t>ATM application will display an error message when the user enters an invalid option</t>
+  </si>
+  <si>
+    <t>ATM application will display an error message when the entered data does not meet the required format</t>
+  </si>
+  <si>
+    <t>ATM application will not modify account data when a transaction fails</t>
+  </si>
+  <si>
+    <t>ATM application will allow the user to retry an operation after a recoverable error</t>
+  </si>
+  <si>
+    <t>ATM application will terminate the current transaction when a critical error prevents the transaction from continuing</t>
+  </si>
+  <si>
+    <t>ATM application will return the user to an appropriate menu after handling a recoverable error</t>
+  </si>
+  <si>
+    <t>ATM application will display the main menu after successful PIN authentication</t>
+  </si>
+  <si>
+    <t>The main menu will provide options for the available ATM functions</t>
+  </si>
+  <si>
+    <t>ATM application will allow the user to select a function from the main menu</t>
+  </si>
+  <si>
+    <t>ATM application will navigate the user to the selected function</t>
+  </si>
+  <si>
+    <t>ATM application will allow the user to return to the main menu after completing or cancelling a transaction</t>
+  </si>
+  <si>
+    <t>ATM application will display an error message when the user selects an unavailable menu option</t>
+  </si>
+  <si>
+    <t>ATM application will allow the user to exit ATM session from the main menu</t>
+  </si>
+  <si>
+    <t>ATM application will allow the user to create a new PIN</t>
+  </si>
+  <si>
+    <t>ATM application will display the user's transaction history</t>
+  </si>
+  <si>
+    <t>ATM application will display the transaction receipt information</t>
+  </si>
+  <si>
+    <t>ATM application will return the card to the user when the session ends</t>
+  </si>
+  <si>
+    <t>Error Message</t>
+  </si>
+  <si>
+    <t>Login</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -154,6 +714,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF0D0D0D"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -175,26 +741,27 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -475,135 +1042,833 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D100"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="14.453125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="55.1796875" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="45.90625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="14.36328125" style="1" customWidth="1"/>
-    <col min="5" max="16384" width="8.7265625" style="1"/>
+    <col min="1" max="1" width="14.453125" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="55.1796875" style="5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="45.90625" style="4" customWidth="1"/>
+    <col min="4" max="4" width="14.36328125" style="4" customWidth="1"/>
+    <col min="5" max="16384" width="8.7265625" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="2" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="29" x14ac:dyDescent="0.35">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="5" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="29" x14ac:dyDescent="0.35">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="5" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="29" x14ac:dyDescent="0.35">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="3"/>
-      <c r="D4" s="4"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
     </row>
     <row r="5" spans="1:4" ht="29" x14ac:dyDescent="0.35">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="3"/>
-      <c r="D5" s="4"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
     </row>
     <row r="6" spans="1:4" ht="29" x14ac:dyDescent="0.35">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="3"/>
-      <c r="D6" s="4"/>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
     </row>
     <row r="7" spans="1:4" ht="29" x14ac:dyDescent="0.35">
-      <c r="A7" s="1" t="s">
+      <c r="A7" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="3"/>
-      <c r="D7" s="4"/>
+      <c r="C7" s="1"/>
+      <c r="D7" s="1"/>
     </row>
     <row r="8" spans="1:4" ht="29" x14ac:dyDescent="0.35">
-      <c r="A8" s="1" t="s">
+      <c r="A8" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="3"/>
-      <c r="D8" s="4"/>
+      <c r="C8" s="1"/>
+      <c r="D8" s="1"/>
     </row>
     <row r="9" spans="1:4" ht="29" x14ac:dyDescent="0.35">
-      <c r="A9" s="1" t="s">
+      <c r="A9" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="3"/>
-      <c r="D9" s="4"/>
+      <c r="C9" s="1"/>
+      <c r="D9" s="1"/>
     </row>
     <row r="10" spans="1:4" ht="29" x14ac:dyDescent="0.35">
-      <c r="A10" s="1" t="s">
+      <c r="A10" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C10" s="3"/>
-      <c r="D10" s="4"/>
+      <c r="C10" s="1"/>
+      <c r="D10" s="1"/>
     </row>
     <row r="11" spans="1:4" ht="29" x14ac:dyDescent="0.35">
-      <c r="A11" s="1" t="s">
+      <c r="A11" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C11" s="3"/>
-      <c r="D11" s="4"/>
+      <c r="C11" s="1"/>
+      <c r="D11" s="1"/>
     </row>
     <row r="12" spans="1:4" ht="29" x14ac:dyDescent="0.35">
-      <c r="A12" s="1" t="s">
+      <c r="A12" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="5" t="s">
         <v>28</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" s="7" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A14" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A15" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A16" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A17" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A18" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A19" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A20" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A21" s="7" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A22" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A23" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A24" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A25" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A26" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A27" s="7" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A28" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A29" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="B29" s="5" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A30" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A31" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B31" s="5" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A32" s="7" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A33" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A34" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="B34" s="5" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A35" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A36" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="B36" s="5" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A37" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="B37" s="5" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A38" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="B38" s="5" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A39" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="B39" s="5" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A40" s="6" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A41" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="B41" s="5" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A42" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B42" s="5" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A43" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="B43" s="5" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A44" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="B44" s="5" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A45" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="B45" s="5" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A46" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="B46" s="5" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A47" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B47" s="5" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A48" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="B48" s="5" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A49" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="B49" s="5" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A50" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="B50" s="5" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A51" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="B51" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A52" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="B52" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="C52" s="4" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A53" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="B53" s="5" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A54" s="6" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A55" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="B55" s="5" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A56" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="B56" s="5" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A57" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="B57" s="5" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A58" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="B58" s="5" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A59" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="B59" s="5" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A60" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="B60" s="5" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A61" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="B61" s="5" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A62" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="B62" s="5" t="s">
+        <v>178</v>
+      </c>
+      <c r="C62" s="4" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A63" s="6" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A64" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="B64" s="5" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A65" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="B65" s="5" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A66" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="B66" s="5" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A67" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="B67" s="5" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A68" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="B68" s="5" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A69" s="7" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A70" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="B70" s="5" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A71" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="B71" s="5" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A72" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="B72" s="5" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A73" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="B73" s="5" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A74" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="B74" s="5" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A75" s="6" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A76" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="B76" s="5" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A77" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="B77" s="5" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A78" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="B78" s="5" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A79" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="B79" s="5" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A80" s="6" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A81" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="B81" s="5" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A82" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="B82" s="5" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A83" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="B83" s="5" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A84" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="B84" s="5" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A85" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="B85" s="5" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A86" s="6" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A87" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="B87" s="5" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A88" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="B88" s="5" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A89" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="B89" s="5" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A90" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="B90" s="5" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A91" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="B91" s="5" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A92" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="B92" s="5" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A93" s="6" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A94" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="B94" s="5" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A95" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="B95" s="5" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A96" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="B96" s="5" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A97" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="B97" s="5" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A98" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="B98" s="5" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A99" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="B99" s="5" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A100" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="B100" s="5" t="s">
+        <v>207</v>
       </c>
     </row>
   </sheetData>
@@ -614,7 +1879,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{736B2B27-1B39-44F2-80F0-178DDCA64A23}">
-  <dimension ref="A3:B4"/>
+  <dimension ref="A3:B15"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.26953125" customWidth="1"/>
@@ -637,6 +1902,94 @@
         <v>3</v>
       </c>
     </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>76</v>
+      </c>
+      <c r="B5" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>78</v>
+      </c>
+      <c r="B6" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>80</v>
+      </c>
+      <c r="B7" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>116</v>
+      </c>
+      <c r="B8" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>117</v>
+      </c>
+      <c r="B9" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>119</v>
+      </c>
+      <c r="B10" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>121</v>
+      </c>
+      <c r="B11" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>123</v>
+      </c>
+      <c r="B12" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>125</v>
+      </c>
+      <c r="B13" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>127</v>
+      </c>
+      <c r="B14" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>130</v>
+      </c>
+      <c r="B15" t="s">
+        <v>129</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>